<commit_message>
script to extract qualitatively CL
</commit_message>
<xml_diff>
--- a/Qualitative_inspection.xlsx
+++ b/Qualitative_inspection.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\CT_Data_PSI\FR54\2023_COELY_postmortem\preliminary_inspection\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git_repos\01_Python\postmortem_coely\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FFA1633-61B0-40F1-9FFC-FD5C0635AE86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80285510-C53E-4D02-8BFB-7004AE13E0D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="39">
   <si>
     <t>operation cond</t>
   </si>
@@ -754,6 +754,9 @@
       <c r="D9" t="s">
         <v>38</v>
       </c>
+      <c r="E9" t="s">
+        <v>38</v>
+      </c>
       <c r="H9" t="s">
         <v>38</v>
       </c>

</xml_diff>